<commit_message>
run x1 no hole
</commit_message>
<xml_diff>
--- a/experiments/results/abp/cplex-mip-abp.xlsx
+++ b/experiments/results/abp/cplex-mip-abp.xlsx
@@ -1,19 +1,20 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="abp_x0.5" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="abp_x0.5_has_hole" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="abp_x0.75" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="abp_x0.75_has_hole" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="abp_x1" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="abp_x1.25" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet name="abp_x1.5" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="abp_x0.5" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="abp_x0.5_no_hole" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="abp_x0.75" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="abp_x0.75_no_hole" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="abp_x1" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="abp_x1.25" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="abp_x1.5" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="abp_x1_no_hole" sheetId="8" state="visible" r:id="rId8"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -23,13 +24,16 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="1">
+  <fonts count="2">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <b val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -40,7 +44,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -48,12 +52,21 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin"/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -423,52 +436,52 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>File</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>Problem</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>Time limit (s)</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>Worker count</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>Target value</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>Lower bound</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>Upper bound</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>Best span</t>
         </is>
       </c>
-      <c r="I1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>Time consumed (s)</t>
         </is>
       </c>
-      <c r="J1" t="inlineStr">
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>Optimal found</t>
         </is>
@@ -511,11 +524,11 @@
         </is>
       </c>
       <c r="H2" t="n">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>58.62</t>
+          <t>2.14</t>
         </is>
       </c>
       <c r="J2" t="inlineStr">
@@ -565,7 +578,7 @@
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>2.73</t>
+          <t>1.71</t>
         </is>
       </c>
       <c r="J3" t="inlineStr">
@@ -615,7 +628,7 @@
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>0.66</t>
+          <t>1.04</t>
         </is>
       </c>
       <c r="J4" t="inlineStr">
@@ -665,7 +678,7 @@
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>1800.01</t>
+          <t>1802.24</t>
         </is>
       </c>
       <c r="J5" t="inlineStr"/>
@@ -711,7 +724,7 @@
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>0.85</t>
+          <t>1.33</t>
         </is>
       </c>
       <c r="J6" t="inlineStr">
@@ -761,7 +774,7 @@
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>1802.39</t>
+          <t>1800.01</t>
         </is>
       </c>
       <c r="J7" t="inlineStr"/>
@@ -807,14 +820,10 @@
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>376.12</t>
-        </is>
-      </c>
-      <c r="J8" t="inlineStr">
-        <is>
-          <t>x</t>
-        </is>
-      </c>
+          <t>1800.10</t>
+        </is>
+      </c>
+      <c r="J8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -857,7 +866,7 @@
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>1800.28</t>
+          <t>1802.64</t>
         </is>
       </c>
       <c r="J9" t="inlineStr"/>
@@ -899,14 +908,18 @@
         </is>
       </c>
       <c r="H10" t="n">
-        <v>38</v>
+        <v>33</v>
       </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t>1800.02</t>
-        </is>
-      </c>
-      <c r="J10" t="inlineStr"/>
+          <t>334.44</t>
+        </is>
+      </c>
+      <c r="J10" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -945,14 +958,18 @@
         </is>
       </c>
       <c r="H11" t="n">
-        <v>41</v>
+        <v>34</v>
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>1800.01</t>
-        </is>
-      </c>
-      <c r="J11" t="inlineStr"/>
+          <t>43.50</t>
+        </is>
+      </c>
+      <c r="J11" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -995,7 +1012,7 @@
       </c>
       <c r="I12" t="inlineStr">
         <is>
-          <t>96.65</t>
+          <t>3.57</t>
         </is>
       </c>
       <c r="J12" t="inlineStr">
@@ -1045,7 +1062,7 @@
       </c>
       <c r="I13" t="inlineStr">
         <is>
-          <t>554.46</t>
+          <t>228.17</t>
         </is>
       </c>
       <c r="J13" t="inlineStr">
@@ -1097,7 +1114,7 @@
       </c>
       <c r="I14" t="inlineStr">
         <is>
-          <t>1800.05</t>
+          <t>1803.96</t>
         </is>
       </c>
       <c r="J14" t="inlineStr"/>
@@ -1145,7 +1162,7 @@
       </c>
       <c r="I15" t="inlineStr">
         <is>
-          <t>1800.05</t>
+          <t>1804.07</t>
         </is>
       </c>
       <c r="J15" t="inlineStr"/>
@@ -1193,7 +1210,7 @@
       </c>
       <c r="I16" t="inlineStr">
         <is>
-          <t>1800.76</t>
+          <t>1802.46</t>
         </is>
       </c>
       <c r="J16" t="inlineStr"/>
@@ -1241,7 +1258,7 @@
       </c>
       <c r="I17" t="inlineStr">
         <is>
-          <t>1800.90</t>
+          <t>1801.67</t>
         </is>
       </c>
       <c r="J17" t="inlineStr"/>
@@ -1282,17 +1299,19 @@
           <t>247</t>
         </is>
       </c>
-      <c r="H18" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+      <c r="H18" t="n">
+        <v>226</v>
       </c>
       <c r="I18" t="inlineStr">
         <is>
-          <t>1800.05</t>
-        </is>
-      </c>
-      <c r="J18" t="inlineStr"/>
+          <t>1093.21</t>
+        </is>
+      </c>
+      <c r="J18" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -1337,7 +1356,7 @@
       </c>
       <c r="I19" t="inlineStr">
         <is>
-          <t>1801.57</t>
+          <t>1800.69</t>
         </is>
       </c>
       <c r="J19" t="inlineStr"/>
@@ -1378,17 +1397,19 @@
           <t>273</t>
         </is>
       </c>
-      <c r="H20" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+      <c r="H20" t="n">
+        <v>130</v>
       </c>
       <c r="I20" t="inlineStr">
         <is>
-          <t>1800.23</t>
-        </is>
-      </c>
-      <c r="J20" t="inlineStr"/>
+          <t>613.84</t>
+        </is>
+      </c>
+      <c r="J20" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -1433,7 +1454,7 @@
       </c>
       <c r="I21" t="inlineStr">
         <is>
-          <t>1801.27</t>
+          <t>1800.13</t>
         </is>
       </c>
       <c r="J21" t="inlineStr"/>
@@ -1474,14 +1495,12 @@
           <t>331</t>
         </is>
       </c>
-      <c r="H22" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+      <c r="H22" t="n">
+        <v>330</v>
       </c>
       <c r="I22" t="inlineStr">
         <is>
-          <t>1800.70</t>
+          <t>1802.51</t>
         </is>
       </c>
       <c r="J22" t="inlineStr"/>
@@ -1529,7 +1548,7 @@
       </c>
       <c r="I23" t="inlineStr">
         <is>
-          <t>1800.11</t>
+          <t>1803.27</t>
         </is>
       </c>
       <c r="J23" t="inlineStr"/>
@@ -1570,14 +1589,12 @@
           <t>342</t>
         </is>
       </c>
-      <c r="H24" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+      <c r="H24" t="n">
+        <v>340</v>
       </c>
       <c r="I24" t="inlineStr">
         <is>
-          <t>1801.15</t>
+          <t>1802.37</t>
         </is>
       </c>
       <c r="J24" t="inlineStr"/>
@@ -1625,7 +1642,7 @@
       </c>
       <c r="I25" t="inlineStr">
         <is>
-          <t>1800.48</t>
+          <t>1800.05</t>
         </is>
       </c>
       <c r="J25" t="inlineStr"/>
@@ -1645,52 +1662,52 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>File</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>Problem</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>Time limit (s)</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>Worker count</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>Target value</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>Lower bound</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>Upper bound</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>Best span</t>
         </is>
       </c>
-      <c r="I1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>Time consumed (s)</t>
         </is>
       </c>
-      <c r="J1" t="inlineStr">
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>Optimal found</t>
         </is>
@@ -1733,11 +1750,11 @@
         </is>
       </c>
       <c r="H2" t="n">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>2.14</t>
+          <t>58.62</t>
         </is>
       </c>
       <c r="J2" t="inlineStr">
@@ -1787,7 +1804,7 @@
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>1.71</t>
+          <t>2.73</t>
         </is>
       </c>
       <c r="J3" t="inlineStr">
@@ -1837,7 +1854,7 @@
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>1.04</t>
+          <t>0.66</t>
         </is>
       </c>
       <c r="J4" t="inlineStr">
@@ -1887,7 +1904,7 @@
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>1802.24</t>
+          <t>1800.01</t>
         </is>
       </c>
       <c r="J5" t="inlineStr"/>
@@ -1933,7 +1950,7 @@
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>1.33</t>
+          <t>0.85</t>
         </is>
       </c>
       <c r="J6" t="inlineStr">
@@ -1983,7 +2000,7 @@
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>1800.01</t>
+          <t>1802.39</t>
         </is>
       </c>
       <c r="J7" t="inlineStr"/>
@@ -2029,10 +2046,14 @@
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>1800.10</t>
-        </is>
-      </c>
-      <c r="J8" t="inlineStr"/>
+          <t>376.12</t>
+        </is>
+      </c>
+      <c r="J8" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -2075,7 +2096,7 @@
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>1802.64</t>
+          <t>1800.28</t>
         </is>
       </c>
       <c r="J9" t="inlineStr"/>
@@ -2117,18 +2138,14 @@
         </is>
       </c>
       <c r="H10" t="n">
-        <v>33</v>
+        <v>38</v>
       </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t>334.44</t>
-        </is>
-      </c>
-      <c r="J10" t="inlineStr">
-        <is>
-          <t>x</t>
-        </is>
-      </c>
+          <t>1800.02</t>
+        </is>
+      </c>
+      <c r="J10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -2167,18 +2184,14 @@
         </is>
       </c>
       <c r="H11" t="n">
-        <v>34</v>
+        <v>41</v>
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>43.50</t>
-        </is>
-      </c>
-      <c r="J11" t="inlineStr">
-        <is>
-          <t>x</t>
-        </is>
-      </c>
+          <t>1800.01</t>
+        </is>
+      </c>
+      <c r="J11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -2221,7 +2234,7 @@
       </c>
       <c r="I12" t="inlineStr">
         <is>
-          <t>3.57</t>
+          <t>96.65</t>
         </is>
       </c>
       <c r="J12" t="inlineStr">
@@ -2271,7 +2284,7 @@
       </c>
       <c r="I13" t="inlineStr">
         <is>
-          <t>228.17</t>
+          <t>554.46</t>
         </is>
       </c>
       <c r="J13" t="inlineStr">
@@ -2323,7 +2336,7 @@
       </c>
       <c r="I14" t="inlineStr">
         <is>
-          <t>1803.96</t>
+          <t>1800.05</t>
         </is>
       </c>
       <c r="J14" t="inlineStr"/>
@@ -2371,7 +2384,7 @@
       </c>
       <c r="I15" t="inlineStr">
         <is>
-          <t>1804.07</t>
+          <t>1800.05</t>
         </is>
       </c>
       <c r="J15" t="inlineStr"/>
@@ -2419,7 +2432,7 @@
       </c>
       <c r="I16" t="inlineStr">
         <is>
-          <t>1802.46</t>
+          <t>1800.76</t>
         </is>
       </c>
       <c r="J16" t="inlineStr"/>
@@ -2467,7 +2480,7 @@
       </c>
       <c r="I17" t="inlineStr">
         <is>
-          <t>1801.67</t>
+          <t>1800.90</t>
         </is>
       </c>
       <c r="J17" t="inlineStr"/>
@@ -2508,19 +2521,17 @@
           <t>247</t>
         </is>
       </c>
-      <c r="H18" t="n">
-        <v>226</v>
+      <c r="H18" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
       </c>
       <c r="I18" t="inlineStr">
         <is>
-          <t>1093.21</t>
-        </is>
-      </c>
-      <c r="J18" t="inlineStr">
-        <is>
-          <t>x</t>
-        </is>
-      </c>
+          <t>1800.05</t>
+        </is>
+      </c>
+      <c r="J18" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -2565,7 +2576,7 @@
       </c>
       <c r="I19" t="inlineStr">
         <is>
-          <t>1800.69</t>
+          <t>1801.57</t>
         </is>
       </c>
       <c r="J19" t="inlineStr"/>
@@ -2606,19 +2617,17 @@
           <t>273</t>
         </is>
       </c>
-      <c r="H20" t="n">
-        <v>130</v>
+      <c r="H20" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
       </c>
       <c r="I20" t="inlineStr">
         <is>
-          <t>613.84</t>
-        </is>
-      </c>
-      <c r="J20" t="inlineStr">
-        <is>
-          <t>x</t>
-        </is>
-      </c>
+          <t>1800.23</t>
+        </is>
+      </c>
+      <c r="J20" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -2663,7 +2672,7 @@
       </c>
       <c r="I21" t="inlineStr">
         <is>
-          <t>1800.13</t>
+          <t>1801.27</t>
         </is>
       </c>
       <c r="J21" t="inlineStr"/>
@@ -2704,12 +2713,14 @@
           <t>331</t>
         </is>
       </c>
-      <c r="H22" t="n">
-        <v>330</v>
+      <c r="H22" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
       </c>
       <c r="I22" t="inlineStr">
         <is>
-          <t>1802.51</t>
+          <t>1800.70</t>
         </is>
       </c>
       <c r="J22" t="inlineStr"/>
@@ -2757,7 +2768,7 @@
       </c>
       <c r="I23" t="inlineStr">
         <is>
-          <t>1803.27</t>
+          <t>1800.11</t>
         </is>
       </c>
       <c r="J23" t="inlineStr"/>
@@ -2798,12 +2809,14 @@
           <t>342</t>
         </is>
       </c>
-      <c r="H24" t="n">
-        <v>340</v>
+      <c r="H24" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
       </c>
       <c r="I24" t="inlineStr">
         <is>
-          <t>1802.37</t>
+          <t>1801.15</t>
         </is>
       </c>
       <c r="J24" t="inlineStr"/>
@@ -2851,7 +2864,7 @@
       </c>
       <c r="I25" t="inlineStr">
         <is>
-          <t>1800.05</t>
+          <t>1800.48</t>
         </is>
       </c>
       <c r="J25" t="inlineStr"/>
@@ -2871,52 +2884,52 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>File</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>Problem</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>Time limit (s)</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>Worker count</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>Target value</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>Lower bound</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>Upper bound</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>Best span</t>
         </is>
       </c>
-      <c r="I1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>Time consumed (s)</t>
         </is>
       </c>
-      <c r="J1" t="inlineStr">
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>Optimal found</t>
         </is>
@@ -2959,11 +2972,11 @@
         </is>
       </c>
       <c r="H2" t="n">
-        <v>15</v>
+        <v>12</v>
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>44.02</t>
+          <t>3.35</t>
         </is>
       </c>
       <c r="J2" t="inlineStr">
@@ -3013,7 +3026,7 @@
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>12.32</t>
+          <t>2.07</t>
         </is>
       </c>
       <c r="J3" t="inlineStr">
@@ -3063,7 +3076,7 @@
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>3.93</t>
+          <t>1.15</t>
         </is>
       </c>
       <c r="J4" t="inlineStr">
@@ -3113,14 +3126,10 @@
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>1087.56</t>
-        </is>
-      </c>
-      <c r="J5" t="inlineStr">
-        <is>
-          <t>x</t>
-        </is>
-      </c>
+          <t>1800.01</t>
+        </is>
+      </c>
+      <c r="J5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -3163,7 +3172,7 @@
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>10.50</t>
+          <t>1.13</t>
         </is>
       </c>
       <c r="J6" t="inlineStr">
@@ -3213,10 +3222,14 @@
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>1800.03</t>
-        </is>
-      </c>
-      <c r="J7" t="inlineStr"/>
+          <t>4.57</t>
+        </is>
+      </c>
+      <c r="J7" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -3259,7 +3272,7 @@
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>280.17</t>
+          <t>2.69</t>
         </is>
       </c>
       <c r="J8" t="inlineStr">
@@ -3309,7 +3322,7 @@
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>1800.01</t>
+          <t>1801.88</t>
         </is>
       </c>
       <c r="J9" t="inlineStr"/>
@@ -3350,17 +3363,19 @@
           <t>63</t>
         </is>
       </c>
-      <c r="H10" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+      <c r="H10" t="n">
+        <v>51</v>
       </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t>1800.01</t>
-        </is>
-      </c>
-      <c r="J10" t="inlineStr"/>
+          <t>327.34</t>
+        </is>
+      </c>
+      <c r="J10" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -3399,14 +3414,18 @@
         </is>
       </c>
       <c r="H11" t="n">
-        <v>72</v>
+        <v>52</v>
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>1800.02</t>
-        </is>
-      </c>
-      <c r="J11" t="inlineStr"/>
+          <t>88.92</t>
+        </is>
+      </c>
+      <c r="J11" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -3445,14 +3464,18 @@
         </is>
       </c>
       <c r="H12" t="n">
-        <v>81</v>
+        <v>76</v>
       </c>
       <c r="I12" t="inlineStr">
         <is>
-          <t>1800.01</t>
-        </is>
-      </c>
-      <c r="J12" t="inlineStr"/>
+          <t>4.40</t>
+        </is>
+      </c>
+      <c r="J12" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -3495,10 +3518,14 @@
       </c>
       <c r="I13" t="inlineStr">
         <is>
-          <t>1800.03</t>
-        </is>
-      </c>
-      <c r="J13" t="inlineStr"/>
+          <t>1418.97</t>
+        </is>
+      </c>
+      <c r="J13" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -3543,7 +3570,7 @@
       </c>
       <c r="I14" t="inlineStr">
         <is>
-          <t>1800.18</t>
+          <t>1800.09</t>
         </is>
       </c>
       <c r="J14" t="inlineStr"/>
@@ -3591,7 +3618,7 @@
       </c>
       <c r="I15" t="inlineStr">
         <is>
-          <t>1800.37</t>
+          <t>1800.09</t>
         </is>
       </c>
       <c r="J15" t="inlineStr"/>
@@ -3639,7 +3666,7 @@
       </c>
       <c r="I16" t="inlineStr">
         <is>
-          <t>1800.04</t>
+          <t>1802.29</t>
         </is>
       </c>
       <c r="J16" t="inlineStr"/>
@@ -3687,7 +3714,7 @@
       </c>
       <c r="I17" t="inlineStr">
         <is>
-          <t>1801.31</t>
+          <t>1802.80</t>
         </is>
       </c>
       <c r="J17" t="inlineStr"/>
@@ -3728,14 +3755,12 @@
           <t>370</t>
         </is>
       </c>
-      <c r="H18" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+      <c r="H18" t="n">
+        <v>365</v>
       </c>
       <c r="I18" t="inlineStr">
         <is>
-          <t>1800.06</t>
+          <t>1800.12</t>
         </is>
       </c>
       <c r="J18" t="inlineStr"/>
@@ -3783,7 +3808,7 @@
       </c>
       <c r="I19" t="inlineStr">
         <is>
-          <t>1801.06</t>
+          <t>1800.16</t>
         </is>
       </c>
       <c r="J19" t="inlineStr"/>
@@ -3824,17 +3849,19 @@
           <t>409</t>
         </is>
       </c>
-      <c r="H20" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+      <c r="H20" t="n">
+        <v>195</v>
       </c>
       <c r="I20" t="inlineStr">
         <is>
-          <t>1800.08</t>
-        </is>
-      </c>
-      <c r="J20" t="inlineStr"/>
+          <t>1330.52</t>
+        </is>
+      </c>
+      <c r="J20" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -3879,7 +3906,7 @@
       </c>
       <c r="I21" t="inlineStr">
         <is>
-          <t>1802.05</t>
+          <t>1801.20</t>
         </is>
       </c>
       <c r="J21" t="inlineStr"/>
@@ -3927,7 +3954,7 @@
       </c>
       <c r="I22" t="inlineStr">
         <is>
-          <t>1801.58</t>
+          <t>1800.18</t>
         </is>
       </c>
       <c r="J22" t="inlineStr"/>
@@ -3975,7 +4002,7 @@
       </c>
       <c r="I23" t="inlineStr">
         <is>
-          <t>1800.15</t>
+          <t>1816.15</t>
         </is>
       </c>
       <c r="J23" t="inlineStr"/>
@@ -4023,7 +4050,7 @@
       </c>
       <c r="I24" t="inlineStr">
         <is>
-          <t>1804.08</t>
+          <t>1803.96</t>
         </is>
       </c>
       <c r="J24" t="inlineStr"/>
@@ -4071,7 +4098,7 @@
       </c>
       <c r="I25" t="inlineStr">
         <is>
-          <t>1800.09</t>
+          <t>1806.52</t>
         </is>
       </c>
       <c r="J25" t="inlineStr"/>
@@ -4091,52 +4118,52 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>File</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>Problem</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>Time limit (s)</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>Worker count</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>Target value</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>Lower bound</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>Upper bound</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>Best span</t>
         </is>
       </c>
-      <c r="I1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>Time consumed (s)</t>
         </is>
       </c>
-      <c r="J1" t="inlineStr">
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>Optimal found</t>
         </is>
@@ -4179,11 +4206,11 @@
         </is>
       </c>
       <c r="H2" t="n">
-        <v>12</v>
+        <v>15</v>
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>3.35</t>
+          <t>44.02</t>
         </is>
       </c>
       <c r="J2" t="inlineStr">
@@ -4233,7 +4260,7 @@
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>2.07</t>
+          <t>12.32</t>
         </is>
       </c>
       <c r="J3" t="inlineStr">
@@ -4283,7 +4310,7 @@
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>1.15</t>
+          <t>3.93</t>
         </is>
       </c>
       <c r="J4" t="inlineStr">
@@ -4333,10 +4360,14 @@
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>1800.01</t>
-        </is>
-      </c>
-      <c r="J5" t="inlineStr"/>
+          <t>1087.56</t>
+        </is>
+      </c>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -4379,7 +4410,7 @@
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>1.13</t>
+          <t>10.50</t>
         </is>
       </c>
       <c r="J6" t="inlineStr">
@@ -4429,14 +4460,10 @@
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>4.57</t>
-        </is>
-      </c>
-      <c r="J7" t="inlineStr">
-        <is>
-          <t>x</t>
-        </is>
-      </c>
+          <t>1800.03</t>
+        </is>
+      </c>
+      <c r="J7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -4479,7 +4506,7 @@
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>2.69</t>
+          <t>280.17</t>
         </is>
       </c>
       <c r="J8" t="inlineStr">
@@ -4529,7 +4556,7 @@
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>1801.88</t>
+          <t>1800.01</t>
         </is>
       </c>
       <c r="J9" t="inlineStr"/>
@@ -4570,19 +4597,17 @@
           <t>63</t>
         </is>
       </c>
-      <c r="H10" t="n">
-        <v>51</v>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
       </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t>327.34</t>
-        </is>
-      </c>
-      <c r="J10" t="inlineStr">
-        <is>
-          <t>x</t>
-        </is>
-      </c>
+          <t>1800.01</t>
+        </is>
+      </c>
+      <c r="J10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -4621,18 +4646,14 @@
         </is>
       </c>
       <c r="H11" t="n">
-        <v>52</v>
+        <v>72</v>
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>88.92</t>
-        </is>
-      </c>
-      <c r="J11" t="inlineStr">
-        <is>
-          <t>x</t>
-        </is>
-      </c>
+          <t>1800.02</t>
+        </is>
+      </c>
+      <c r="J11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -4671,18 +4692,14 @@
         </is>
       </c>
       <c r="H12" t="n">
-        <v>76</v>
+        <v>81</v>
       </c>
       <c r="I12" t="inlineStr">
         <is>
-          <t>4.40</t>
-        </is>
-      </c>
-      <c r="J12" t="inlineStr">
-        <is>
-          <t>x</t>
-        </is>
-      </c>
+          <t>1800.01</t>
+        </is>
+      </c>
+      <c r="J12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -4725,14 +4742,10 @@
       </c>
       <c r="I13" t="inlineStr">
         <is>
-          <t>1418.97</t>
-        </is>
-      </c>
-      <c r="J13" t="inlineStr">
-        <is>
-          <t>x</t>
-        </is>
-      </c>
+          <t>1800.03</t>
+        </is>
+      </c>
+      <c r="J13" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -4777,7 +4790,7 @@
       </c>
       <c r="I14" t="inlineStr">
         <is>
-          <t>1800.09</t>
+          <t>1800.18</t>
         </is>
       </c>
       <c r="J14" t="inlineStr"/>
@@ -4825,7 +4838,7 @@
       </c>
       <c r="I15" t="inlineStr">
         <is>
-          <t>1800.09</t>
+          <t>1800.37</t>
         </is>
       </c>
       <c r="J15" t="inlineStr"/>
@@ -4873,7 +4886,7 @@
       </c>
       <c r="I16" t="inlineStr">
         <is>
-          <t>1802.29</t>
+          <t>1800.04</t>
         </is>
       </c>
       <c r="J16" t="inlineStr"/>
@@ -4921,7 +4934,7 @@
       </c>
       <c r="I17" t="inlineStr">
         <is>
-          <t>1802.80</t>
+          <t>1801.31</t>
         </is>
       </c>
       <c r="J17" t="inlineStr"/>
@@ -4962,12 +4975,14 @@
           <t>370</t>
         </is>
       </c>
-      <c r="H18" t="n">
-        <v>365</v>
+      <c r="H18" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
       </c>
       <c r="I18" t="inlineStr">
         <is>
-          <t>1800.12</t>
+          <t>1800.06</t>
         </is>
       </c>
       <c r="J18" t="inlineStr"/>
@@ -5015,7 +5030,7 @@
       </c>
       <c r="I19" t="inlineStr">
         <is>
-          <t>1800.16</t>
+          <t>1801.06</t>
         </is>
       </c>
       <c r="J19" t="inlineStr"/>
@@ -5056,19 +5071,17 @@
           <t>409</t>
         </is>
       </c>
-      <c r="H20" t="n">
-        <v>195</v>
+      <c r="H20" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
       </c>
       <c r="I20" t="inlineStr">
         <is>
-          <t>1330.52</t>
-        </is>
-      </c>
-      <c r="J20" t="inlineStr">
-        <is>
-          <t>x</t>
-        </is>
-      </c>
+          <t>1800.08</t>
+        </is>
+      </c>
+      <c r="J20" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -5113,7 +5126,7 @@
       </c>
       <c r="I21" t="inlineStr">
         <is>
-          <t>1801.20</t>
+          <t>1802.05</t>
         </is>
       </c>
       <c r="J21" t="inlineStr"/>
@@ -5161,7 +5174,7 @@
       </c>
       <c r="I22" t="inlineStr">
         <is>
-          <t>1800.18</t>
+          <t>1801.58</t>
         </is>
       </c>
       <c r="J22" t="inlineStr"/>
@@ -5209,7 +5222,7 @@
       </c>
       <c r="I23" t="inlineStr">
         <is>
-          <t>1816.15</t>
+          <t>1800.15</t>
         </is>
       </c>
       <c r="J23" t="inlineStr"/>
@@ -5257,7 +5270,7 @@
       </c>
       <c r="I24" t="inlineStr">
         <is>
-          <t>1803.96</t>
+          <t>1804.08</t>
         </is>
       </c>
       <c r="J24" t="inlineStr"/>
@@ -5305,7 +5318,7 @@
       </c>
       <c r="I25" t="inlineStr">
         <is>
-          <t>1806.52</t>
+          <t>1800.09</t>
         </is>
       </c>
       <c r="J25" t="inlineStr"/>
@@ -5325,52 +5338,52 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>File</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>Problem</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>Time limit (s)</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>Worker count</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>Target value</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>Lower bound</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>Upper bound</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>Best span</t>
         </is>
       </c>
-      <c r="I1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>Time consumed (s)</t>
         </is>
       </c>
-      <c r="J1" t="inlineStr">
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>Optimal found</t>
         </is>
@@ -6559,52 +6572,52 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>File</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>Problem</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>Time limit (s)</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>Worker count</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>Target value</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>Lower bound</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>Upper bound</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>Best span</t>
         </is>
       </c>
-      <c r="I1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>Time consumed (s)</t>
         </is>
       </c>
-      <c r="J1" t="inlineStr">
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>Optimal found</t>
         </is>
@@ -7795,52 +7808,52 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>File</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>Problem</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>Time limit (s)</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>Worker count</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>Target value</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>Lower bound</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>Upper bound</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>Best span</t>
         </is>
       </c>
-      <c r="I1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>Time consumed (s)</t>
         </is>
       </c>
-      <c r="J1" t="inlineStr">
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>Optimal found</t>
         </is>
@@ -9006,6 +9019,1228 @@
       <c r="I25" t="inlineStr">
         <is>
           <t>1800.85</t>
+        </is>
+      </c>
+      <c r="J25" t="inlineStr"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:J25"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>File</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Problem</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Time limit (s)</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Worker count</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Target value</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>Lower bound</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>Upper bound</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>Best span</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>Time consumed (s)</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>Optimal found</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>A-pores_1.txt</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>A-pores_1.mtx.rnd</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>1800</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>30</t>
+        </is>
+      </c>
+      <c r="H2" t="n">
+        <v>23</v>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>567.42</t>
+        </is>
+      </c>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>B-ibm32.txt</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>B-ibm32.mtx.rnd</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>1800</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>9</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>32</t>
+        </is>
+      </c>
+      <c r="H3" t="n">
+        <v>29</v>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>1800.01</t>
+        </is>
+      </c>
+      <c r="J3" t="inlineStr"/>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>C-bcspwr01.txt</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>C-bcspwr01.mtx.rnd</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>1800</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>17</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>18</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>39</t>
+        </is>
+      </c>
+      <c r="H4" t="n">
+        <v>38</v>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>1389.39</t>
+        </is>
+      </c>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>D-bcsstk01.txt</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>D-bcsstk01.mtx.rnd</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>1800</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>9</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>48</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>1800.01</t>
+        </is>
+      </c>
+      <c r="J5" t="inlineStr"/>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>E-bcspwr02.txt</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>E-bcspwr02.mtx.rnd</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>1800</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>21</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>22</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>49</t>
+        </is>
+      </c>
+      <c r="H6" t="n">
+        <v>45</v>
+      </c>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>136.97</t>
+        </is>
+      </c>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>F-curtis54.txt</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>F-curtis54.mtx.rnd</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>1800</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>13</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>14</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>54</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>1800.19</t>
+        </is>
+      </c>
+      <c r="J7" t="inlineStr"/>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>G-will57.txt</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>G-will57.mtx.rnd</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>1800</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>13</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>14</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>57</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>1800.01</t>
+        </is>
+      </c>
+      <c r="J8" t="inlineStr"/>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>H-impcol_b.txt</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>H-impcol_b.mtx.rnd</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>1800</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>9</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>59</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>1800.02</t>
+        </is>
+      </c>
+      <c r="J9" t="inlineStr"/>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>I-ash85.txt</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>I-ash85.mtx.rnd</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>1800</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>23</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>24</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>85</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I10" t="inlineStr">
+        <is>
+          <t>1800.45</t>
+        </is>
+      </c>
+      <c r="J10" t="inlineStr"/>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>J-nos4.txt</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>J-nos4.mtx.rnd</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>1800</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>35</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>36</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>100</t>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I11" t="inlineStr">
+        <is>
+          <t>1800.03</t>
+        </is>
+      </c>
+      <c r="J11" t="inlineStr"/>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>K-dwt__234.txt</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>K-dwt__234.mtx.rnd</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>1800</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>51</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>52</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>117</t>
+        </is>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I12" t="inlineStr">
+        <is>
+          <t>1800.02</t>
+        </is>
+      </c>
+      <c r="J12" t="inlineStr"/>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>L-bcspwr03.txt</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>L-bcspwr03.mtx.rnd</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>1800</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>39</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>40</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>118</t>
+        </is>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I13" t="inlineStr">
+        <is>
+          <t>1800.02</t>
+        </is>
+      </c>
+      <c r="J13" t="inlineStr"/>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>M-bcsstk06.txt</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>M-bcsstk06.mtx.rnd</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>1800</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>34</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>35</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>420</t>
+        </is>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I14" t="inlineStr">
+        <is>
+          <t>1800.11</t>
+        </is>
+      </c>
+      <c r="J14" t="inlineStr"/>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>N-bcsstk07.txt</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>N-bcsstk07.mtx.rnd</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>1800</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>34</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>35</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>420</t>
+        </is>
+      </c>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I15" t="inlineStr">
+        <is>
+          <t>1800.20</t>
+        </is>
+      </c>
+      <c r="J15" t="inlineStr"/>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>O-impcol_d.txt</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>O-impcol_d.mtx.rnd</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>1800</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>120</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>121</t>
+        </is>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>425</t>
+        </is>
+      </c>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I16" t="inlineStr">
+        <is>
+          <t>1800.11</t>
+        </is>
+      </c>
+      <c r="J16" t="inlineStr"/>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>P-can__445.txt</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>P-can__445.mtx.rnd</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>1800</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>90</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>91</t>
+        </is>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>445</t>
+        </is>
+      </c>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I17" t="inlineStr">
+        <is>
+          <t>1803.03</t>
+        </is>
+      </c>
+      <c r="J17" t="inlineStr"/>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>Q-494_bus.txt</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>Q-494_bus.mtx.rnd</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>1800</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>227</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>228</t>
+        </is>
+      </c>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>494</t>
+        </is>
+      </c>
+      <c r="H18" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I18" t="inlineStr">
+        <is>
+          <t>1800.16</t>
+        </is>
+      </c>
+      <c r="J18" t="inlineStr"/>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>R-dwt__503.txt</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>R-dwt__503.mtx.rnd</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>1800</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>63</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>64</t>
+        </is>
+      </c>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>503</t>
+        </is>
+      </c>
+      <c r="H19" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I19" t="inlineStr">
+        <is>
+          <t>1807.10</t>
+        </is>
+      </c>
+      <c r="J19" t="inlineStr"/>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>S-sherman4.txt</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>S-sherman4.mtx.rnd</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>1800</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>261</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>262</t>
+        </is>
+      </c>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>546</t>
+        </is>
+      </c>
+      <c r="H20" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I20" t="inlineStr">
+        <is>
+          <t>1800.22</t>
+        </is>
+      </c>
+      <c r="J20" t="inlineStr"/>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>T-dwt__592.txt</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>T-dwt__592.mtx.rnd</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>1800</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>113</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>114</t>
+        </is>
+      </c>
+      <c r="G21" t="inlineStr">
+        <is>
+          <t>592</t>
+        </is>
+      </c>
+      <c r="H21" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I21" t="inlineStr">
+        <is>
+          <t>1801.78</t>
+        </is>
+      </c>
+      <c r="J21" t="inlineStr"/>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>U-662_bus.txt</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>U-662_bus.mtx.rnd</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>1800</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>220</t>
+        </is>
+      </c>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>221</t>
+        </is>
+      </c>
+      <c r="G22" t="inlineStr">
+        <is>
+          <t>662</t>
+        </is>
+      </c>
+      <c r="H22" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I22" t="inlineStr">
+        <is>
+          <t>1804.08</t>
+        </is>
+      </c>
+      <c r="J22" t="inlineStr"/>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>V-nos6.txt</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>V-nos6.mtx.rnd</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>1800</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>329</t>
+        </is>
+      </c>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>330</t>
+        </is>
+      </c>
+      <c r="G23" t="inlineStr">
+        <is>
+          <t>675</t>
+        </is>
+      </c>
+      <c r="H23" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I23" t="inlineStr">
+        <is>
+          <t>1800.29</t>
+        </is>
+      </c>
+      <c r="J23" t="inlineStr"/>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>W-685_bus.txt</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>W-685_bus.mtx.rnd</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>1800</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>136</t>
+        </is>
+      </c>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>137</t>
+        </is>
+      </c>
+      <c r="G24" t="inlineStr">
+        <is>
+          <t>685</t>
+        </is>
+      </c>
+      <c r="H24" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I24" t="inlineStr">
+        <is>
+          <t>1800.59</t>
+        </is>
+      </c>
+      <c r="J24" t="inlineStr"/>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>X-can__715.txt</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>X-can__715.mtx.rnd</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>1800</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>116</t>
+        </is>
+      </c>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>117</t>
+        </is>
+      </c>
+      <c r="G25" t="inlineStr">
+        <is>
+          <t>715</t>
+        </is>
+      </c>
+      <c r="H25" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I25" t="inlineStr">
+        <is>
+          <t>1800.40</t>
         </is>
       </c>
       <c r="J25" t="inlineStr"/>

</xml_diff>